<commit_message>
fix: clean excel templates and rebuild charts visually
- 模板清洗全部从第 1 行开始（固定品牌/日期/小红书TOP15 标题清除，由导出器
  动态写入每个 Sheet 标题）；TEMPLATE_VERSION 改文档自定义属性（不再写 A1000，
  used range 不再扩到 1000 行）
- write_table 数据行统一 font/border/alignment/交替填充/行高；KOL Top20 行样式
  一致
- 品牌日趋势写表头（系列名来自表头）、日期轴写文本 ISO；热门帖子/活动热帖
  URL 写超链接
- 活动平台图表引用从第 5 行开始；周期对比/情感/归属图表按数据重建，空章节
  不画误导图；ROI Sheet 来自受控模板（无 ROI 移除、不创建裸白表）
- 新增测试：无示例残留、KOL 样式一致、图表真实引用、used range、ROI 条件
</commit_message>
<xml_diff>
--- a/backend/app/agent_artifacts/templates/brand_report_v3.xlsx
+++ b/backend/app/agent_artifacts/templates/brand_report_v3.xlsx
@@ -15,9 +15,7 @@
     <sheet name="舆情洞察" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="方法论" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
-  <definedNames>
-    <definedName name="TEMPLATE_VERSION">'综合概览'!$A$1000</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -588,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1000"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.35"/>
   <cols>
     <col width="34" customWidth="1" style="12" min="1" max="1"/>
@@ -598,47 +596,19 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" s="12">
-      <c r="A1" s="13" t="inlineStr">
-        <is>
-          <t>昊来了 品牌社交媒体表现分析报告</t>
-        </is>
-      </c>
+      <c r="A1" s="13" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>分析周期</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-30 至 2026-07-30</t>
-        </is>
-      </c>
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>数据来源</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>DataTap 聆媒洞察 MCP (小红书 + 抖音)</t>
-        </is>
-      </c>
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>搜索方式</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>关键词搜索: "昊来了"</t>
-        </is>
-      </c>
+      <c r="A4" s="1" t="n"/>
+      <c r="B4" s="2" t="n"/>
     </row>
     <row r="5"/>
     <row r="6">
@@ -758,18 +728,6 @@
       <c r="A28" s="4" t="n"/>
       <c r="B28" s="4" t="n"/>
       <c r="C28" s="22" t="n"/>
-    </row>
-    <row r="1000">
-      <c r="A1000" t="inlineStr">
-        <is>
-          <t>gate-c-v1</t>
-        </is>
-      </c>
-      <c r="B1000" t="inlineStr">
-        <is>
-          <t>template_version</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -797,11 +755,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="17.7" customHeight="1" s="12">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>内容情感分布 (按平台)</t>
-        </is>
-      </c>
+      <c r="A1" s="15" t="n"/>
     </row>
     <row r="2"/>
     <row r="3">
@@ -900,11 +854,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="17.7" customHeight="1" s="12">
-      <c r="A1" s="16" t="inlineStr">
-        <is>
-          <t>每日声量与互动趋势 (2026-06-30 至 2026-07-30)</t>
-        </is>
-      </c>
+      <c r="A1" s="16" t="n"/>
     </row>
     <row r="2"/>
     <row r="3">
@@ -1128,11 +1078,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="17.7" customHeight="1" s="12">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>内容类型分布</t>
-        </is>
-      </c>
+      <c r="A1" s="17" t="n"/>
     </row>
     <row r="2"/>
     <row r="3">
@@ -1277,11 +1223,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="17.7" customHeight="1" s="12">
-      <c r="A1" s="18" t="inlineStr">
-        <is>
-          <t>发帖用户地域分布 TOP 20</t>
-        </is>
-      </c>
+      <c r="A1" s="18" t="n"/>
     </row>
     <row r="2"/>
     <row r="3">
@@ -1436,11 +1378,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="17.7" customHeight="1" s="12">
-      <c r="A1" s="19" t="inlineStr">
-        <is>
-          <t>小红书热门帖子 TOP 15 (品牌相关, 按互动数排序)</t>
-        </is>
-      </c>
+      <c r="A1" s="19" t="n"/>
     </row>
     <row r="2"/>
     <row r="3">
@@ -1921,11 +1859,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="17.7" customHeight="1" s="12">
-      <c r="A1" s="20" t="inlineStr">
-        <is>
-          <t>舆情洞察与内容主题分析</t>
-        </is>
-      </c>
+      <c r="A1" s="20" t="n"/>
     </row>
     <row r="2"/>
     <row r="3">
@@ -2056,11 +1990,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="17.7" customHeight="1" s="12">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>数据说明与方法论</t>
-        </is>
-      </c>
+      <c r="A1" s="21" t="n"/>
     </row>
     <row r="2"/>
     <row r="3">

</xml_diff>